<commit_message>
Sua grid cha con  va phan trang lai
</commit_message>
<xml_diff>
--- a/modules/work_assignment/views/report/approve/template-excel.xlsx
+++ b/modules/work_assignment/views/report/approve/template-excel.xlsx
@@ -49,7 +49,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -59,13 +59,27 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <name val="Calibri"/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -108,22 +122,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,144 +490,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="32.36328125" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="9.6328125" customWidth="1"/>
-    <col min="6" max="6" width="12.90625" customWidth="1"/>
+    <col min="1" max="1" width="6" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12" style="2" customWidth="1"/>
+    <col min="3" max="3" width="32.36328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17" style="2" customWidth="1"/>
+    <col min="5" max="5" width="9.6328125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.90625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="125.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
-    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.5">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.4">
+      <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>